<commit_message>
Update documentation links to use the master branch for example references
</commit_message>
<xml_diff>
--- a/examples/output/usage-workbook.xlsx
+++ b/examples/output/usage-workbook.xlsx
@@ -2,12 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr date1904="false"/>
+  <workbookProtection lockStructure="1"/>
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" r:id="rId3" sheetId="1"/>
+    <sheet name="Summary" r:id="rId4" sheetId="2"/>
   </sheets>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId5"/>
+  </pivotCaches>
 </workbook>
 </file>
 
@@ -133,10 +138,23 @@
 </styleSheet>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="UTF-8"?>
+<pivotCacheDefinition:http://schemas.openxmlformats.org/spreadsheetml/2006/main xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="" refreshOnLoad="1" updatedBy="DotnetPoi" createdVersion="3" minRefreshableVersion="3" recordCount="0" upgradeOnRefresh="1"><cacheSource type="worksheet"><worksheetSource ref="A3:D6" sheet="Invoice"/></cacheSource></pivotCacheDefinition:http://schemas.openxmlformats.org/spreadsheetml/2006/main>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="UTF-8"?>
+<pivotCacheRecords:http://schemas.openxmlformats.org/spreadsheetml/2006/main count="0"/>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="UTF-8"?>
+<pivotTableDefinition:http://schemas.openxmlformats.org/spreadsheetml/2006/main xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="0" dataCaption="Values" multipleFieldFilters="0" indent="0" createdVersion="3" minRefreshableVersion="3" updatedVersion="3" itemPrintTitles="1" useAutoFormatting="1" applyNumberFormats="0" applyWidthHeightFormats="1" applyAlignmentFormats="0" applyPatternFormats="0" applyFontFormats="0" applyBorderFormats="0"><location ref="A1:B2" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/><pivotFields count="4"><pivotField showAll="0" axis="axisRow"/><pivotField showAll="0"/><pivotField showAll="0"/><pivotField showAll="0" dataField="1"/></pivotFields><rowFields count="1"><field x="0"/></rowFields><dataFields count="1"><dataField name="Sum of Field4" fld="3" subtotal="sum"/></dataFields><pivotTableStyleInfo name="PivotStyleLight16" showLastColumn="1" showColStripes="0" showRowStripes="0" showColHeaders="1" showRowHeaders="1"/></pivotTableDefinition:http://schemas.openxmlformats.org/spreadsheetml/2006/main>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <cols>
     <col min="1" max="1" width="24.00" customWidth="true"/>
     <col min="2" max="2" width="14.00" customWidth="true"/>
@@ -225,6 +243,16 @@
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
+  <autoFilter ref="A3:D6"/>
+  <pageMargins bottom="0.7500" footer="0.3000" header="0.3000" left="0.7000" right="0.7000" top="0.7500"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData/>
   <pageMargins bottom="0.7500" footer="0.3000" header="0.3000" left="0.7000" right="0.7000" top="0.7500"/>
 </worksheet>
 </file>
</xml_diff>